<commit_message>
🎓 Slice organismes de formation 2026-10-09
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -93,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -102,6 +102,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P2" headerRowCount="1">
-  <autoFilter ref="A1:P2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P3" headerRowCount="1">
+  <autoFilter ref="A1:P3"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -530,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -556,14 +559,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="39" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
@@ -573,7 +576,7 @@
     <col width="27" customWidth="1" min="12" max="12"/>
     <col width="27" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
@@ -662,72 +665,138 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="inlineStr"/>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr"/>
-      <c r="E2" s="5" t="inlineStr"/>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-10
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P3" headerRowCount="1">
-  <autoFilter ref="A1:P3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P4" headerRowCount="1">
+  <autoFilter ref="A1:P4"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,27 +665,27 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -700,17 +700,17 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr"/>
@@ -724,79 +724,145 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr"/>
+      <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="6" t="inlineStr"/>
+      <c r="N3" s="6" t="inlineStr"/>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O3" s="6" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P3" s="6" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-12
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -104,10 +104,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P4" headerRowCount="1">
-  <autoFilter ref="A1:P4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P5" headerRowCount="1">
+  <autoFilter ref="A1:P5"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -571,10 +571,10 @@
     <col width="25" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="59" customWidth="1" min="10" max="10"/>
     <col width="27" customWidth="1" min="11" max="11"/>
     <col width="27" customWidth="1" min="12" max="12"/>
-    <col width="27" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
@@ -665,32 +665,24 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -700,169 +692,251 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr"/>
-      <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
-      <c r="N2" s="5" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>11922496392</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>90386961800012</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>11756597175</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>80360838900026</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>COORPACADEMY FRANCE</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>PARIS 09</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>486807</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>2713</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>Energie, génie climatique</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr"/>
-      <c r="L3" s="6" t="inlineStr"/>
-      <c r="M3" s="6" t="inlineStr"/>
-      <c r="N3" s="6" t="inlineStr"/>
-      <c r="O3" s="6" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>426616</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr"/>
+      <c r="L3" s="7" t="inlineStr"/>
+      <c r="M3" s="7" t="inlineStr"/>
+      <c r="N3" s="7" t="inlineStr"/>
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>introuvable</t>
         </is>
       </c>
-      <c r="P3" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-09 11:12:58</t>
+      <c r="P3" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
+      <c r="N4" s="5" t="inlineStr"/>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M5" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N5" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O5" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-13
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P5" headerRowCount="1">
-  <autoFilter ref="A1:P5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P6" headerRowCount="1">
+  <autoFilter ref="A1:P6"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -568,7 +568,7 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="59" customWidth="1" min="10" max="10"/>
@@ -665,59 +665,67 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr"/>
-      <c r="E2" s="5" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
+          <t>https://www.aftral.com</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>contact@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
@@ -732,39 +740,31 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -774,58 +774,74 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr"/>
-      <c r="L3" s="7" t="inlineStr"/>
-      <c r="M3" s="7" t="inlineStr"/>
-      <c r="N3" s="7" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P3" s="7" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -840,17 +856,17 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr"/>
@@ -864,79 +880,145 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="inlineStr"/>
+      <c r="M5" s="7" t="inlineStr"/>
+      <c r="N5" s="7" t="inlineStr"/>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P5" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M5" s="7" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O5" s="7" t="inlineStr">
+      <c r="O6" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P5" s="7" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-14
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -104,10 +104,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P6" headerRowCount="1">
-  <autoFilter ref="A1:P6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P8" headerRowCount="1">
+  <autoFilter ref="A1:P8"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -571,12 +571,12 @@
     <col width="29" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="59" customWidth="1" min="10" max="10"/>
-    <col width="27" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="29" customWidth="1" min="11" max="11"/>
     <col width="27" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
@@ -665,29 +665,21 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>11750091675</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>30540504500017</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
+          <t>SAFRAN</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr">
         <is>
           <t>11</t>
@@ -695,153 +687,141 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>formation;apprentissage;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>293734</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Transport, manutention, magasinage</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>https://www.aftral.com</t>
-        </is>
-      </c>
-      <c r="L2" s="6" t="inlineStr">
-        <is>
-          <t>dpd@aftral.com</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>dpd@aftral.com</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13 11:34:14</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>82690030969</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>95550398200014</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>11920012692</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>55202467100091</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>368655</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>https://www.desautel.fr</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>contact@desautel.fr</t>
-        </is>
-      </c>
-      <c r="M3" s="7" t="inlineStr">
-        <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
-        </is>
-      </c>
-      <c r="N3" s="7" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>187508</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>1936</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>https://www.cegos.fr</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O3" s="7" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P3" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-12 11:47:00</t>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
+          <t>AFTRAL</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75847</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>PARIS 09</t>
+          <t>PARIS 17</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -851,174 +831,330 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="5" t="inlineStr"/>
+          <t>Transport, manutention, magasinage</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aftral.com</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>dpd@aftral.com</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>dpd@aftral.com</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>11922496392</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>90386961800012</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>82690030969</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>95550398200014</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>486807</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>2713</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Energie, génie climatique</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr"/>
-      <c r="L5" s="7" t="inlineStr"/>
-      <c r="M5" s="7" t="inlineStr"/>
-      <c r="N5" s="7" t="inlineStr"/>
-      <c r="O5" s="7" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P5" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-09 11:12:58</t>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>368655</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
+          <t>11756597175</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>80360838900026</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>COORPACADEMY FRANCE</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 09</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>426616</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:30:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P7" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L8" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O8" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="P8" s="5" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-15
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P8" headerRowCount="1">
-  <autoFilter ref="A1:P8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P9" headerRowCount="1">
+  <autoFilter ref="A1:P9"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,24 +665,32 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr"/>
-      <c r="E2" s="5" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -692,12 +700,12 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -707,7 +715,7 @@
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr"/>
@@ -720,24 +728,24 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:38</t>
+          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr"/>
@@ -754,76 +762,56 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>187508</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N3" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="6" t="inlineStr"/>
+      <c r="N3" s="6" t="inlineStr"/>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:39</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11750091675</t>
+          <t>11920012692</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>30540504500017</t>
+          <t>55202467100091</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
           <t>11</t>
@@ -831,37 +819,37 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>formation;apprentissage;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>293734</t>
+          <t>187508</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Transport, manutention, magasinage</t>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>https://www.aftral.com</t>
+          <t>https://www.cegos.fr</t>
         </is>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
@@ -876,66 +864,74 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13 11:34:14</t>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
+          <t>https://www.aftral.com</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>contact@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
@@ -950,39 +946,31 @@
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -992,58 +980,74 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -1058,17 +1062,17 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr"/>
@@ -1082,79 +1086,145 @@
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
+      <c r="N8" s="5" t="inlineStr"/>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L8" s="7" t="inlineStr">
+      <c r="L9" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N8" s="5" t="inlineStr">
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O8" s="5" t="inlineStr">
+      <c r="O9" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P8" s="5" t="inlineStr">
+      <c r="P9" s="6" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-17
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -104,10 +104,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P9" headerRowCount="1">
-  <autoFilter ref="A1:P9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P10" headerRowCount="1">
+  <autoFilter ref="A1:P10"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
-    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
     <col width="27" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
@@ -665,32 +665,24 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>76310894831</t>
+          <t>11788376778</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>38347481400100</t>
+          <t>83409674500197</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
+          <t>SOCOTEC FORMATION</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -700,114 +692,134 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>182662</t>
+          <t>181212</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Technologies industrielles fondamentales</t>
+          <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
-      <c r="N2" s="5" t="inlineStr"/>
+          <t>https://formation.socotec.fr</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 09:02:13</t>
+          <t>2026-10-17 08:24:44</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>11750082675</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>56208290901190</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>76310894831</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>38347481400100</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>239038</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>182662</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>377</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>http://safran-formation.com</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr"/>
-      <c r="M3" s="6" t="inlineStr"/>
-      <c r="N3" s="6" t="inlineStr"/>
-      <c r="O3" s="6" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>https://www.airbus.com</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr"/>
+      <c r="M3" s="7" t="inlineStr"/>
+      <c r="N3" s="7" t="inlineStr"/>
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>site_sans_email</t>
         </is>
       </c>
-      <c r="P3" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-14 09:23:38</t>
+      <c r="P3" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr"/>
@@ -824,188 +836,176 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>187508</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L4" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
+      <c r="N4" s="5" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:39</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>11750091675</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>30540504500017</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>11920012692</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>55202467100091</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>formation;apprentissage;vae</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>293734</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>2259</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Transport, manutention, magasinage</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>https://www.aftral.com</t>
-        </is>
-      </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>dpd@aftral.com</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>dpd@aftral.com</t>
-        </is>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>187508</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>1936</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>https://www.cegos.fr</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="O5" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P5" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-13 11:34:14</t>
+      <c r="P5" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
-        </is>
-      </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>contact@desautel.fr</t>
+          <t>https://www.aftral.com</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -1020,100 +1020,108 @@
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>11756597175</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>80360838900026</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>82690030969</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>95550398200014</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>426616</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P7" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-10 10:30:20</t>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>368655</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -1128,17 +1136,17 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr"/>
@@ -1152,79 +1160,145 @@
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr"/>
+      <c r="N9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr"/>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M9" s="6" t="inlineStr">
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N9" s="6" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O9" s="6" t="inlineStr">
+      <c r="O10" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P9" s="6" t="inlineStr">
+      <c r="P10" s="5" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-19
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -104,10 +104,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P10" headerRowCount="1">
-  <autoFilter ref="A1:P10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P11" headerRowCount="1">
+  <autoFilter ref="A1:P11"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,168 +665,172 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>11753916975</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>47916313100119</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>147210</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>1043</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="inlineStr"/>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-19 09:44:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
           <t>11788376778</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>83409674500197</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>SOCOTEC FORMATION</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr"/>
-      <c r="E2" s="5" t="inlineStr"/>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>181212</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>1344</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>https://formation.socotec.fr</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr">
         <is>
           <t>formation@socotec.com</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>formation@socotec.com</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>2026-10-17 08:24:44</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>76310894831</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>38347481400100</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>182662</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>377</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>Technologies industrielles fondamentales</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr"/>
-      <c r="M3" s="7" t="inlineStr"/>
-      <c r="N3" s="7" t="inlineStr"/>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>site_sans_email</t>
-        </is>
-      </c>
-      <c r="P3" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -836,12 +840,12 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -851,7 +855,7 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr"/>
@@ -864,441 +868,503 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
+          <t>2026-10-15 09:02:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>11750082675</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>56208290901190</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>SAFRAN</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>239038</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Technologies industrielles fondamentales</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="6" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr"/>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>site_sans_email</t>
+        </is>
+      </c>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
           <t>2026-10-14 09:23:38</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>11920012692</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>55202467100091</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>CEGOS SA</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>187508</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>1936</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N5" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O5" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P5" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
+          <t>11920012692</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>55202467100091</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>187508</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>1936</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cegos.fr</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 09:23:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
           <t>11750091675</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>30540504500017</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>AFTRAL</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>75847</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>PARIS 17</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>formation;apprentissage;vae</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>293734</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>2259</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>Transport, manutention, magasinage</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>https://www.aftral.com</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr">
         <is>
           <t>dpd@aftral.com</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>dpd@aftral.com</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>2026-10-13 11:34:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>82690030969</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>95550398200014</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>368655</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>https://www.desautel.fr</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>contact@desautel.fr</t>
-        </is>
-      </c>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
-        </is>
-      </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P7" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
+          <t>82690030969</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>95550398200014</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>368655</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12 11:47:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
           <t>11756597175</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>80360838900026</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>75009</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>PARIS 09</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>426616</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Formations générales</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="inlineStr"/>
-      <c r="O8" s="5" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="inlineStr">
         <is>
           <t>introuvable</t>
         </is>
       </c>
-      <c r="P8" s="5" t="inlineStr">
+      <c r="P9" s="6" t="inlineStr">
         <is>
           <t>2026-10-10 10:30:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>11922496392</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>90386961800012</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>486807</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>2713</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>Energie, génie climatique</t>
-        </is>
-      </c>
-      <c r="K9" s="7" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr"/>
-      <c r="M9" s="7" t="inlineStr"/>
-      <c r="N9" s="7" t="inlineStr"/>
-      <c r="O9" s="7" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P9" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-09 11:12:58</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr"/>
+      <c r="M10" s="5" t="inlineStr"/>
+      <c r="N10" s="5" t="inlineStr"/>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="L11" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O10" s="5" t="inlineStr">
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P10" s="5" t="inlineStr">
+      <c r="P11" s="6" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-20
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P11" headerRowCount="1">
-  <autoFilter ref="A1:P11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P12" headerRowCount="1">
+  <autoFilter ref="A1:P12"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,87 +665,91 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>11753916975</t>
+          <t>22020084902</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>47916313100119</t>
+          <t>39017462100404</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>147210</t>
+          <t>142980</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>707</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr"/>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
       <c r="L2" s="5" t="inlineStr"/>
       <c r="M2" s="5" t="inlineStr"/>
       <c r="N2" s="5" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19 09:44:56</t>
+          <t>2026-10-20 09:17:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>11788376778</t>
+          <t>11753916975</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>83409674500197</t>
+          <t>47916313100119</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>SOCOTEC FORMATION</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
           <t>11</t>
@@ -758,79 +762,55 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>181212</t>
+          <t>147210</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Electricité, électronique (non compris automatisme et productique)</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>https://formation.socotec.fr</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="N3" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr"/>
+      <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="6" t="inlineStr"/>
+      <c r="N3" s="6" t="inlineStr"/>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-17 08:24:44</t>
+          <t>2026-10-19 09:44:56</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>76310894831</t>
+          <t>11788376778</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>38347481400100</t>
+          <t>83409674500197</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
+          <t>SOCOTEC FORMATION</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -840,59 +820,79 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>182662</t>
+          <t>181212</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Technologies industrielles fondamentales</t>
+          <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="5" t="inlineStr"/>
+          <t>https://formation.socotec.fr</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 09:02:13</t>
+          <t>2026-10-17 08:24:44</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -902,12 +902,12 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr"/>
@@ -930,24 +930,24 @@
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:38</t>
+          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr"/>
@@ -964,76 +964,56 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>187508</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:39</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>11750091675</t>
+          <t>11920012692</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>30540504500017</t>
+          <t>55202467100091</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
       <c r="F7" s="6" t="inlineStr">
         <is>
           <t>11</t>
@@ -1041,37 +1021,37 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>formation;apprentissage;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>293734</t>
+          <t>187508</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Transport, manutention, magasinage</t>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>https://www.aftral.com</t>
+          <t>https://www.cegos.fr</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
@@ -1086,66 +1066,74 @@
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-13 11:34:14</t>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
+          <t>https://www.aftral.com</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>contact@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -1160,39 +1148,31 @@
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1202,58 +1182,74 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr"/>
-      <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="6" t="inlineStr"/>
-      <c r="N9" s="6" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1268,17 +1264,17 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr"/>
@@ -1292,79 +1288,145 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
+      <c r="M11" s="6" t="inlineStr"/>
+      <c r="N11" s="6" t="inlineStr"/>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr"/>
-      <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr">
+      <c r="L12" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M11" s="6" t="inlineStr">
+      <c r="M12" s="5" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N11" s="6" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O11" s="6" t="inlineStr">
+      <c r="O12" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P11" s="6" t="inlineStr">
+      <c r="P12" s="5" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-21
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P12" headerRowCount="1">
-  <autoFilter ref="A1:P12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P13" headerRowCount="1">
+  <autoFilter ref="A1:P13"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -559,16 +559,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
@@ -665,17 +665,17 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>22020084902</t>
+          <t>31590340859</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>39017462100404</t>
+          <t>40073444800022</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>AKSIS</t>
+          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr"/>
@@ -687,127 +687,127 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>formation;bilan</t>
+          <t>formation;apprentissage;bilan</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>142980</t>
+          <t>129603</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>https://www.aksis.fr</t>
-        </is>
-      </c>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr"/>
       <c r="L2" s="5" t="inlineStr"/>
       <c r="M2" s="5" t="inlineStr"/>
       <c r="N2" s="5" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20 09:17:58</t>
+          <t>2026-10-21 09:14:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>11753916975</t>
+          <t>22020084902</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>47916313100119</t>
+          <t>39017462100404</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>147210</t>
+          <t>142980</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>707</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr"/>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
       <c r="L3" s="6" t="inlineStr"/>
       <c r="M3" s="6" t="inlineStr"/>
       <c r="N3" s="6" t="inlineStr"/>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-19 09:44:56</t>
+          <t>2026-10-20 09:17:58</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11788376778</t>
+          <t>11753916975</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>83409674500197</t>
+          <t>47916313100119</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>SOCOTEC FORMATION</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
           <t>11</t>
@@ -820,79 +820,55 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>181212</t>
+          <t>147210</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Electricité, électronique (non compris automatisme et productique)</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>https://formation.socotec.fr</t>
-        </is>
-      </c>
-      <c r="L4" s="7" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
+      <c r="N4" s="5" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17 08:24:44</t>
+          <t>2026-10-19 09:44:56</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>76310894831</t>
+          <t>11788376778</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>38347481400100</t>
+          <t>83409674500197</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
+          <t>SOCOTEC FORMATION</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -902,59 +878,79 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>182662</t>
+          <t>181212</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Technologies industrielles fondamentales</t>
+          <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="inlineStr"/>
-      <c r="M5" s="6" t="inlineStr"/>
-      <c r="N5" s="6" t="inlineStr"/>
+          <t>https://formation.socotec.fr</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-15 09:02:13</t>
+          <t>2026-10-17 08:24:44</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -964,12 +960,12 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -979,7 +975,7 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr"/>
@@ -992,24 +988,24 @@
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:38</t>
+          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr"/>
@@ -1026,76 +1022,56 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>187508</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M7" s="6" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N7" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:39</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>11750091675</t>
+          <t>11920012692</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>30540504500017</t>
+          <t>55202467100091</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="5" t="inlineStr">
         <is>
           <t>11</t>
@@ -1103,37 +1079,37 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>formation;apprentissage;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>293734</t>
+          <t>187508</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Transport, manutention, magasinage</t>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>https://www.aftral.com</t>
+          <t>https://www.cegos.fr</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -1148,66 +1124,74 @@
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13 11:34:14</t>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr"/>
-      <c r="E9" s="6" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
+          <t>https://www.aftral.com</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>contact@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
@@ -1222,39 +1206,31 @@
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1264,58 +1240,74 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr"/>
-      <c r="L10" s="5" t="inlineStr"/>
-      <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1330,17 +1322,17 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr"/>
@@ -1354,79 +1346,145 @@
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr"/>
+      <c r="M12" s="5" t="inlineStr"/>
+      <c r="N12" s="5" t="inlineStr"/>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr"/>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr">
+      <c r="L13" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N12" s="5" t="inlineStr">
+      <c r="N13" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O12" s="5" t="inlineStr">
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P12" s="5" t="inlineStr">
+      <c r="P13" s="6" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-22
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P13" headerRowCount="1">
-  <autoFilter ref="A1:P13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P14" headerRowCount="1">
+  <autoFilter ref="A1:P14"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,75 +665,79 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>31590340859</t>
+          <t>28610102561</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>40073444800022</t>
+          <t>83411160100011</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr"/>
       <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>formation;apprentissage;bilan</t>
+          <t>formation;vae</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>129603</t>
+          <t>128484</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>2756</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr"/>
+          <t>Linguistique</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>https://udd.eu</t>
+        </is>
+      </c>
       <c r="L2" s="5" t="inlineStr"/>
       <c r="M2" s="5" t="inlineStr"/>
       <c r="N2" s="5" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 09:14:55</t>
+          <t>2026-10-22 09:17:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>22020084902</t>
+          <t>31590340859</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>39017462100404</t>
+          <t>40073444800022</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>AKSIS</t>
+          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr"/>
@@ -745,127 +749,127 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>formation;bilan</t>
+          <t>formation;apprentissage;bilan</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>142980</t>
+          <t>129603</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>https://www.aksis.fr</t>
-        </is>
-      </c>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr"/>
       <c r="M3" s="6" t="inlineStr"/>
       <c r="N3" s="6" t="inlineStr"/>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-20 09:17:58</t>
+          <t>2026-10-21 09:14:55</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11753916975</t>
+          <t>22020084902</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>47916313100119</t>
+          <t>39017462100404</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>147210</t>
+          <t>142980</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>707</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr"/>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
       <c r="L4" s="5" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr"/>
       <c r="N4" s="5" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19 09:44:56</t>
+          <t>2026-10-20 09:17:58</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>11788376778</t>
+          <t>11753916975</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>83409674500197</t>
+          <t>47916313100119</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>SOCOTEC FORMATION</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
           <t>11</t>
@@ -878,79 +882,55 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>181212</t>
+          <t>147210</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Electricité, électronique (non compris automatisme et productique)</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>https://formation.socotec.fr</t>
-        </is>
-      </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="6" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr"/>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t>2026-10-17 08:24:44</t>
+          <t>2026-10-19 09:44:56</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>76310894831</t>
+          <t>11788376778</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>38347481400100</t>
+          <t>83409674500197</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
+          <t>SOCOTEC FORMATION</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -960,59 +940,79 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>182662</t>
+          <t>181212</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Technologies industrielles fondamentales</t>
+          <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr"/>
+          <t>https://formation.socotec.fr</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 09:02:13</t>
+          <t>2026-10-17 08:24:44</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -1022,12 +1022,12 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr"/>
@@ -1050,24 +1050,24 @@
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:38</t>
+          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr"/>
@@ -1084,76 +1084,56 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>187508</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
+      <c r="N8" s="5" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:39</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>11750091675</t>
+          <t>11920012692</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>30540504500017</t>
+          <t>55202467100091</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
       <c r="F9" s="6" t="inlineStr">
         <is>
           <t>11</t>
@@ -1161,37 +1141,37 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>formation;apprentissage;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>293734</t>
+          <t>187508</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Transport, manutention, magasinage</t>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>https://www.aftral.com</t>
+          <t>https://www.cegos.fr</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
@@ -1206,66 +1186,74 @@
       </c>
       <c r="P9" s="6" t="inlineStr">
         <is>
-          <t>2026-10-13 11:34:14</t>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
+          <t>https://www.aftral.com</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>contact@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
@@ -1280,39 +1268,31 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1322,58 +1302,74 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr"/>
-      <c r="L11" s="6" t="inlineStr"/>
-      <c r="M11" s="6" t="inlineStr"/>
-      <c r="N11" s="6" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1388,17 +1384,17 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr"/>
@@ -1412,79 +1408,145 @@
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr"/>
+      <c r="M13" s="6" t="inlineStr"/>
+      <c r="N13" s="6" t="inlineStr"/>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr"/>
-      <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr">
+      <c r="L14" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M13" s="6" t="inlineStr">
+      <c r="M14" s="5" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N13" s="6" t="inlineStr">
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O13" s="6" t="inlineStr">
+      <c r="O14" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P13" s="6" t="inlineStr">
+      <c r="P14" s="5" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-23
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -104,10 +104,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P14" headerRowCount="1">
-  <autoFilter ref="A1:P14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P15" headerRowCount="1">
+  <autoFilter ref="A1:P15"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,137 +665,161 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>53351042035</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>83923926600043</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>SIMANGO</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>RENNES</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>119833</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Santé</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>https://simango.fr</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 09:13:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
           <t>28610102561</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>83411160100011</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>UDD</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr"/>
-      <c r="E2" s="5" t="inlineStr"/>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>formation;vae</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>128484</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>2756</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Linguistique</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>https://udd.eu</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
-      <c r="N2" s="5" t="inlineStr"/>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr"/>
+      <c r="M3" s="7" t="inlineStr"/>
+      <c r="N3" s="7" t="inlineStr"/>
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>site_sans_email</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>2026-10-22 09:17:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>31590340859</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>40073444800022</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>formation;apprentissage;bilan</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>129603</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>520</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr"/>
-      <c r="L3" s="6" t="inlineStr"/>
-      <c r="M3" s="6" t="inlineStr"/>
-      <c r="N3" s="6" t="inlineStr"/>
-      <c r="O3" s="6" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P3" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-21 09:14:55</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>22020084902</t>
+          <t>31590340859</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>39017462100404</t>
+          <t>40073444800022</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>AKSIS</t>
+          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr"/>
@@ -807,274 +831,270 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>formation;bilan</t>
+          <t>formation;apprentissage;bilan</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>142980</t>
+          <t>129603</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>https://www.aksis.fr</t>
-        </is>
-      </c>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr"/>
       <c r="L4" s="5" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr"/>
       <c r="N4" s="5" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 09:14:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>22020084902</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>39017462100404</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>formation;bilan</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>142980</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>707</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr"/>
+      <c r="M5" s="7" t="inlineStr"/>
+      <c r="N5" s="7" t="inlineStr"/>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
           <t>site_sans_email</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>2026-10-20 09:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>11753916975</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>47916313100119</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>147210</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>1043</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr"/>
-      <c r="L5" s="6" t="inlineStr"/>
-      <c r="M5" s="6" t="inlineStr"/>
-      <c r="N5" s="6" t="inlineStr"/>
-      <c r="O5" s="6" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P5" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-19 09:44:56</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
+          <t>11753916975</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>47916313100119</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>147210</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>1043</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-19 09:44:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
           <t>11788376778</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>83409674500197</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>SOCOTEC FORMATION</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>181212</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>1344</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>https://formation.socotec.fr</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>formation@socotec.com</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>formation@socotec.com</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="N7" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O7" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="P7" s="7" t="inlineStr">
         <is>
           <t>2026-10-17 08:24:44</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>76310894831</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>38347481400100</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>182662</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>377</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Technologies industrielles fondamentales</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr">
-        <is>
-          <t>site_sans_email</t>
-        </is>
-      </c>
-      <c r="P7" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1084,12 +1104,12 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -1099,7 +1119,7 @@
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr"/>
@@ -1112,441 +1132,503 @@
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
+          <t>2026-10-15 09:02:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>11750082675</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>56208290901190</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>SAFRAN</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>239038</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Technologies industrielles fondamentales</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr"/>
+      <c r="N9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>site_sans_email</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
           <t>2026-10-14 09:23:38</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>11920012692</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>55202467100091</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>CEGOS SA</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr"/>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>187508</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>1936</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N9" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P9" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>11920012692</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>55202467100091</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>187508</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>1936</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cegos.fr</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 09:23:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
           <t>11750091675</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>30540504500017</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>AFTRAL</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>75847</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>PARIS 17</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>formation;apprentissage;vae</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>293734</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>2259</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>Transport, manutention, magasinage</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>https://www.aftral.com</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>dpd@aftral.com</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M11" s="7" t="inlineStr">
         <is>
           <t>dpd@aftral.com</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="N11" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O10" s="5" t="inlineStr">
+      <c r="O11" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P10" s="5" t="inlineStr">
+      <c r="P11" s="7" t="inlineStr">
         <is>
           <t>2026-10-13 11:34:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>82690030969</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>95550398200014</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr"/>
-      <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>368655</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>https://www.desautel.fr</t>
-        </is>
-      </c>
-      <c r="L11" s="7" t="inlineStr">
-        <is>
-          <t>contact@desautel.fr</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
-        </is>
-      </c>
-      <c r="N11" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O11" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P11" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
+          <t>82690030969</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>95550398200014</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>368655</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12 11:47:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
           <t>11756597175</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>80360838900026</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>75009</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>PARIS 09</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>426616</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J13" s="7" t="inlineStr">
         <is>
           <t>Formations générales</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr"/>
-      <c r="L12" s="5" t="inlineStr"/>
-      <c r="M12" s="5" t="inlineStr"/>
-      <c r="N12" s="5" t="inlineStr"/>
-      <c r="O12" s="5" t="inlineStr">
+      <c r="K13" s="7" t="inlineStr"/>
+      <c r="L13" s="7" t="inlineStr"/>
+      <c r="M13" s="7" t="inlineStr"/>
+      <c r="N13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr">
         <is>
           <t>introuvable</t>
         </is>
       </c>
-      <c r="P12" s="5" t="inlineStr">
+      <c r="P13" s="7" t="inlineStr">
         <is>
           <t>2026-10-10 10:30:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>11922496392</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>90386961800012</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>486807</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>2713</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Energie, génie climatique</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr"/>
-      <c r="L13" s="6" t="inlineStr"/>
-      <c r="M13" s="6" t="inlineStr"/>
-      <c r="N13" s="6" t="inlineStr"/>
-      <c r="O13" s="6" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P13" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-09 11:12:58</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr"/>
+      <c r="M14" s="5" t="inlineStr"/>
+      <c r="N14" s="5" t="inlineStr"/>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr"/>
-      <c r="E14" s="5" t="inlineStr"/>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J15" s="7" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K15" s="7" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="M15" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="N15" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr">
+      <c r="O15" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P14" s="5" t="inlineStr">
+      <c r="P15" s="7" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-24
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P15" headerRowCount="1">
-  <autoFilter ref="A1:P15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P16" headerRowCount="1">
+  <autoFilter ref="A1:P16"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,67 +665,59 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>53351042035</t>
+          <t>11754723775</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>83923926600043</t>
+          <t>53014903800719</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>SIMANGO</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>35000</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>RENNES</t>
-        </is>
-      </c>
+          <t>ENVERGURE</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan;vae</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>119833</t>
+          <t>118818</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>858</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Santé</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>https://simango.fr</t>
+          <t>https://www.envergure.eu</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>contact@simango.fr</t>
+          <t>jean.dupont@gmail.com</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+          <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
@@ -740,144 +732,168 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23 09:13:07</t>
+          <t>2026-10-24 08:46:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>28610102561</t>
+          <t>53351042035</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>83411160100011</t>
+          <t>83923926600043</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>UDD</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
+          <t>SIMANGO</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>RENNES</t>
+        </is>
+      </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>formation;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>128484</t>
+          <t>119833</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>2756</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Linguistique</t>
+          <t>Santé</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>https://udd.eu</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr"/>
-      <c r="M3" s="7" t="inlineStr"/>
-      <c r="N3" s="7" t="inlineStr"/>
+          <t>https://simango.fr</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P3" s="7" t="inlineStr">
         <is>
-          <t>2026-10-22 09:17:57</t>
+          <t>2026-10-23 09:13:07</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>31590340859</t>
+          <t>28610102561</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>40073444800022</t>
+          <t>83411160100011</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>formation;apprentissage;bilan</t>
+          <t>formation;vae</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>129603</t>
+          <t>128484</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>2756</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr"/>
+          <t>Linguistique</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>https://udd.eu</t>
+        </is>
+      </c>
       <c r="L4" s="5" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr"/>
       <c r="N4" s="5" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 09:14:55</t>
+          <t>2026-10-22 09:17:57</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>22020084902</t>
+          <t>31590340859</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>39017462100404</t>
+          <t>40073444800022</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>AKSIS</t>
+          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr"/>
@@ -889,127 +905,127 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>formation;bilan</t>
+          <t>formation;apprentissage;bilan</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>142980</t>
+          <t>129603</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>https://www.aksis.fr</t>
-        </is>
-      </c>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr"/>
       <c r="L5" s="7" t="inlineStr"/>
       <c r="M5" s="7" t="inlineStr"/>
       <c r="N5" s="7" t="inlineStr"/>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>2026-10-20 09:17:58</t>
+          <t>2026-10-21 09:14:55</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>11753916975</t>
+          <t>22020084902</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>47916313100119</t>
+          <t>39017462100404</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>147210</t>
+          <t>142980</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>707</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr"/>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
       <c r="L6" s="5" t="inlineStr"/>
       <c r="M6" s="5" t="inlineStr"/>
       <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19 09:44:56</t>
+          <t>2026-10-20 09:17:58</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>11788376778</t>
+          <t>11753916975</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>83409674500197</t>
+          <t>47916313100119</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>SOCOTEC FORMATION</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
           <t>11</t>
@@ -1022,79 +1038,55 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>181212</t>
+          <t>147210</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Electricité, électronique (non compris automatisme et productique)</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>https://formation.socotec.fr</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
+      <c r="M7" s="7" t="inlineStr"/>
+      <c r="N7" s="7" t="inlineStr"/>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>2026-10-17 08:24:44</t>
+          <t>2026-10-19 09:44:56</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>76310894831</t>
+          <t>11788376778</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>38347481400100</t>
+          <t>83409674500197</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
+          <t>SOCOTEC FORMATION</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1104,59 +1096,79 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>182662</t>
+          <t>181212</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Technologies industrielles fondamentales</t>
+          <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="inlineStr"/>
+          <t>https://formation.socotec.fr</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 09:02:13</t>
+          <t>2026-10-17 08:24:44</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1166,12 +1178,12 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
@@ -1181,7 +1193,7 @@
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr"/>
@@ -1194,24 +1206,24 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:38</t>
+          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr"/>
@@ -1228,76 +1240,56 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>187508</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L10" s="6" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr"/>
+      <c r="M10" s="5" t="inlineStr"/>
+      <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:39</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>11750091675</t>
+          <t>11920012692</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>30540504500017</t>
+          <t>55202467100091</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="inlineStr"/>
       <c r="F11" s="7" t="inlineStr">
         <is>
           <t>11</t>
@@ -1305,37 +1297,37 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>formation;apprentissage;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>293734</t>
+          <t>187508</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Transport, manutention, magasinage</t>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>https://www.aftral.com</t>
+          <t>https://www.cegos.fr</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -1350,66 +1342,74 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>2026-10-13 11:34:14</t>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
+          <t>https://www.aftral.com</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>contact@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
@@ -1424,39 +1424,31 @@
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="inlineStr"/>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1466,58 +1458,74 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="inlineStr"/>
-      <c r="L13" s="7" t="inlineStr"/>
-      <c r="M13" s="7" t="inlineStr"/>
-      <c r="N13" s="7" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O13" s="7" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1532,17 +1540,17 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr"/>
@@ -1556,79 +1564,145 @@
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr"/>
+      <c r="N15" s="7" t="inlineStr"/>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr"/>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M15" s="7" t="inlineStr">
+      <c r="M16" s="5" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O15" s="7" t="inlineStr">
+      <c r="O16" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P15" s="7" t="inlineStr">
+      <c r="P16" s="5" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-26
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P16" headerRowCount="1">
-  <autoFilter ref="A1:P16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P17" headerRowCount="1">
+  <autoFilter ref="A1:P17"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -572,8 +572,8 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="31" customWidth="1" min="11" max="11"/>
+    <col width="31" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
@@ -665,17 +665,17 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>11754723775</t>
+          <t>11756068975</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>53014903800719</t>
+          <t>79935188700077</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>ENVERGURE</t>
+          <t>MARIANNE FORMATION</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr"/>
@@ -687,37 +687,37 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>formation;bilan;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>118818</t>
+          <t>116400</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>858</t>
+          <t>2036</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
+          <t>Enseignement, formation</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>https://www.envergure.eu</t>
+          <t>https://marianne-education.fr</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>jean.dupont@gmail.com</t>
+          <t>contact@marianne-education.fr</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
+          <t>contact@marianne-education.fr</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
@@ -732,74 +732,66 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24 08:46:35</t>
+          <t>2026-10-26 09:56:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>53351042035</t>
+          <t>11754723775</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>83923926600043</t>
+          <t>53014903800719</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>SIMANGO</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>35000</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>RENNES</t>
-        </is>
-      </c>
+          <t>ENVERGURE</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan;vae</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>119833</t>
+          <t>118818</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>858</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Santé</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>https://simango.fr</t>
+          <t>https://www.envergure.eu</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>contact@simango.fr</t>
+          <t>jean.dupont@gmail.com</t>
         </is>
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+          <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
@@ -814,144 +806,168 @@
       </c>
       <c r="P3" s="7" t="inlineStr">
         <is>
-          <t>2026-10-23 09:13:07</t>
+          <t>2026-10-24 08:46:35</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>28610102561</t>
+          <t>53351042035</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>83411160100011</t>
+          <t>83923926600043</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>UDD</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
+          <t>SIMANGO</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>RENNES</t>
+        </is>
+      </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>formation;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>128484</t>
+          <t>119833</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>2756</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Linguistique</t>
+          <t>Santé</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>https://udd.eu</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="5" t="inlineStr"/>
+          <t>https://simango.fr</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 09:17:57</t>
+          <t>2026-10-23 09:13:07</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>31590340859</t>
+          <t>28610102561</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>40073444800022</t>
+          <t>83411160100011</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr"/>
       <c r="E5" s="7" t="inlineStr"/>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>formation;apprentissage;bilan</t>
+          <t>formation;vae</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>129603</t>
+          <t>128484</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>2756</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr"/>
+          <t>Linguistique</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>https://udd.eu</t>
+        </is>
+      </c>
       <c r="L5" s="7" t="inlineStr"/>
       <c r="M5" s="7" t="inlineStr"/>
       <c r="N5" s="7" t="inlineStr"/>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>2026-10-21 09:14:55</t>
+          <t>2026-10-22 09:17:57</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>22020084902</t>
+          <t>31590340859</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>39017462100404</t>
+          <t>40073444800022</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>AKSIS</t>
+          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr"/>
@@ -963,127 +979,127 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>formation;bilan</t>
+          <t>formation;apprentissage;bilan</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>142980</t>
+          <t>129603</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>https://www.aksis.fr</t>
-        </is>
-      </c>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr"/>
       <c r="L6" s="5" t="inlineStr"/>
       <c r="M6" s="5" t="inlineStr"/>
       <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20 09:17:58</t>
+          <t>2026-10-21 09:14:55</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>11753916975</t>
+          <t>22020084902</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>47916313100119</t>
+          <t>39017462100404</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>147210</t>
+          <t>142980</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>707</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr"/>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
       <c r="L7" s="7" t="inlineStr"/>
       <c r="M7" s="7" t="inlineStr"/>
       <c r="N7" s="7" t="inlineStr"/>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19 09:44:56</t>
+          <t>2026-10-20 09:17:58</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>11788376778</t>
+          <t>11753916975</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>83409674500197</t>
+          <t>47916313100119</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>SOCOTEC FORMATION</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
           <t>11</t>
@@ -1096,79 +1112,55 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>181212</t>
+          <t>147210</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Electricité, électronique (non compris automatisme et productique)</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>https://formation.socotec.fr</t>
-        </is>
-      </c>
-      <c r="L8" s="6" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
+      <c r="N8" s="5" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17 08:24:44</t>
+          <t>2026-10-19 09:44:56</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>76310894831</t>
+          <t>11788376778</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>38347481400100</t>
+          <t>83409674500197</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
+          <t>SOCOTEC FORMATION</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1178,59 +1170,79 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>182662</t>
+          <t>181212</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Technologies industrielles fondamentales</t>
+          <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="inlineStr"/>
-      <c r="M9" s="7" t="inlineStr"/>
-      <c r="N9" s="7" t="inlineStr"/>
+          <t>https://formation.socotec.fr</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 09:02:13</t>
+          <t>2026-10-17 08:24:44</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1240,12 +1252,12 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1255,7 +1267,7 @@
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr"/>
@@ -1268,24 +1280,24 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:38</t>
+          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr"/>
@@ -1302,76 +1314,56 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>187508</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L11" s="6" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M11" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N11" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr"/>
+      <c r="N11" s="7" t="inlineStr"/>
       <c r="O11" s="7" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:39</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>11750091675</t>
+          <t>11920012692</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>30540504500017</t>
+          <t>55202467100091</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
       <c r="F12" s="5" t="inlineStr">
         <is>
           <t>11</t>
@@ -1379,37 +1371,37 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>formation;apprentissage;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>293734</t>
+          <t>187508</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Transport, manutention, magasinage</t>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>https://www.aftral.com</t>
+          <t>https://www.cegos.fr</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
@@ -1424,66 +1416,74 @@
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13 11:34:14</t>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr"/>
-      <c r="E13" s="7" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
+          <t>https://www.aftral.com</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>contact@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -1498,39 +1498,31 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1540,58 +1532,74 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K14" s="5" t="inlineStr"/>
-      <c r="L14" s="5" t="inlineStr"/>
-      <c r="M14" s="5" t="inlineStr"/>
-      <c r="N14" s="5" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -1606,17 +1614,17 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr"/>
@@ -1630,79 +1638,145 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr"/>
+      <c r="M16" s="5" t="inlineStr"/>
+      <c r="N16" s="5" t="inlineStr"/>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr"/>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M17" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N16" s="5" t="inlineStr">
+      <c r="N17" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O16" s="5" t="inlineStr">
+      <c r="O17" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P16" s="5" t="inlineStr">
+      <c r="P17" s="7" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-27
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P17" headerRowCount="1">
-  <autoFilter ref="A1:P17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P18" headerRowCount="1">
+  <autoFilter ref="A1:P18"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,21 +665,29 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>11756068975</t>
+          <t>11921529392</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>79935188700077</t>
+          <t>48276116000019</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>MARIANNE FORMATION</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr"/>
-      <c r="E2" s="5" t="inlineStr"/>
+          <t>ORSYS</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>92044</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>PUTEAUX</t>
+        </is>
+      </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
           <t>11</t>
@@ -692,32 +700,32 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>116400</t>
+          <t>116153</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>2036</t>
+          <t>1795</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Enseignement, formation</t>
+          <t>Spécialités plurivalentes des échanges et de la gestion</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>https://marianne-education.fr</t>
+          <t>https://www.orsys.fr</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>contact@marianne-education.fr</t>
+          <t>contactpresse@orsys.fr</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>contact@marianne-education.fr</t>
+          <t>contactpresse@orsys.fr;psh-accueil@orsys.fr;rgpd@orsys.fr</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
@@ -732,24 +740,24 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26 09:56:33</t>
+          <t>2026-10-27 09:42:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>11754723775</t>
+          <t>11756068975</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>53014903800719</t>
+          <t>79935188700077</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>ENVERGURE</t>
+          <t>MARIANNE FORMATION</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr"/>
@@ -761,37 +769,37 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>formation;bilan;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>118818</t>
+          <t>116400</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>858</t>
+          <t>2036</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Formations générales</t>
+          <t>Enseignement, formation</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>https://www.envergure.eu</t>
+          <t>https://marianne-education.fr</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>jean.dupont@gmail.com</t>
+          <t>contact@marianne-education.fr</t>
         </is>
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
+          <t>contact@marianne-education.fr</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
@@ -806,74 +814,66 @@
       </c>
       <c r="P3" s="7" t="inlineStr">
         <is>
-          <t>2026-10-24 08:46:35</t>
+          <t>2026-10-26 09:56:33</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>53351042035</t>
+          <t>11754723775</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>83923926600043</t>
+          <t>53014903800719</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>SIMANGO</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>35000</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>RENNES</t>
-        </is>
-      </c>
+          <t>ENVERGURE</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan;vae</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>119833</t>
+          <t>118818</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>858</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Santé</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>https://simango.fr</t>
+          <t>https://www.envergure.eu</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>contact@simango.fr</t>
+          <t>jean.dupont@gmail.com</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+          <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
@@ -888,144 +888,168 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23 09:13:07</t>
+          <t>2026-10-24 08:46:35</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>28610102561</t>
+          <t>53351042035</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>83411160100011</t>
+          <t>83923926600043</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>UDD</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
+          <t>SIMANGO</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>RENNES</t>
+        </is>
+      </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>formation;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>128484</t>
+          <t>119833</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>2756</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Linguistique</t>
+          <t>Santé</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>https://udd.eu</t>
-        </is>
-      </c>
-      <c r="L5" s="7" t="inlineStr"/>
-      <c r="M5" s="7" t="inlineStr"/>
-      <c r="N5" s="7" t="inlineStr"/>
+          <t>https://simango.fr</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>2026-10-22 09:17:57</t>
+          <t>2026-10-23 09:13:07</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>31590340859</t>
+          <t>28610102561</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>40073444800022</t>
+          <t>83411160100011</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>formation;apprentissage;bilan</t>
+          <t>formation;vae</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>129603</t>
+          <t>128484</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>2756</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr"/>
+          <t>Linguistique</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>https://udd.eu</t>
+        </is>
+      </c>
       <c r="L6" s="5" t="inlineStr"/>
       <c r="M6" s="5" t="inlineStr"/>
       <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21 09:14:55</t>
+          <t>2026-10-22 09:17:57</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>22020084902</t>
+          <t>31590340859</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>39017462100404</t>
+          <t>40073444800022</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>AKSIS</t>
+          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr"/>
@@ -1037,127 +1061,127 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>formation;bilan</t>
+          <t>formation;apprentissage;bilan</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>142980</t>
+          <t>129603</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>https://www.aksis.fr</t>
-        </is>
-      </c>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr"/>
       <c r="M7" s="7" t="inlineStr"/>
       <c r="N7" s="7" t="inlineStr"/>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>2026-10-20 09:17:58</t>
+          <t>2026-10-21 09:14:55</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>11753916975</t>
+          <t>22020084902</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>47916313100119</t>
+          <t>39017462100404</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>147210</t>
+          <t>142980</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>707</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr"/>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr"/>
       <c r="N8" s="5" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19 09:44:56</t>
+          <t>2026-10-20 09:17:58</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>11788376778</t>
+          <t>11753916975</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>83409674500197</t>
+          <t>47916313100119</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>SOCOTEC FORMATION</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr"/>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
           <t>11</t>
@@ -1170,79 +1194,55 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>181212</t>
+          <t>147210</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Electricité, électronique (non compris automatisme et productique)</t>
-        </is>
-      </c>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>https://formation.socotec.fr</t>
-        </is>
-      </c>
-      <c r="L9" s="6" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="M9" s="7" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr"/>
+      <c r="N9" s="7" t="inlineStr"/>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-17 08:24:44</t>
+          <t>2026-10-19 09:44:56</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>76310894831</t>
+          <t>11788376778</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>38347481400100</t>
+          <t>83409674500197</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
+          <t>SOCOTEC FORMATION</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1252,59 +1252,79 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>182662</t>
+          <t>181212</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Technologies industrielles fondamentales</t>
+          <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr"/>
-      <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr"/>
+          <t>https://formation.socotec.fr</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 09:02:13</t>
+          <t>2026-10-17 08:24:44</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr"/>
-      <c r="E11" s="7" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1314,12 +1334,12 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -1329,7 +1349,7 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr"/>
@@ -1342,24 +1362,24 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:38</t>
+          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr"/>
@@ -1376,76 +1396,56 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>187508</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr"/>
+      <c r="M12" s="5" t="inlineStr"/>
+      <c r="N12" s="5" t="inlineStr"/>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:39</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>11750091675</t>
+          <t>11920012692</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>30540504500017</t>
+          <t>55202467100091</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="inlineStr"/>
       <c r="F13" s="7" t="inlineStr">
         <is>
           <t>11</t>
@@ -1453,37 +1453,37 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>formation;apprentissage;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>293734</t>
+          <t>187508</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Transport, manutention, magasinage</t>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>https://www.aftral.com</t>
+          <t>https://www.cegos.fr</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -1498,66 +1498,74 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>2026-10-13 11:34:14</t>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr"/>
-      <c r="E14" s="5" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
+          <t>https://www.aftral.com</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>contact@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -1572,39 +1580,31 @@
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="inlineStr"/>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -1614,58 +1614,74 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K15" s="7" t="inlineStr"/>
-      <c r="L15" s="7" t="inlineStr"/>
-      <c r="M15" s="7" t="inlineStr"/>
-      <c r="N15" s="7" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O15" s="7" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1680,17 +1696,17 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr"/>
@@ -1704,79 +1720,145 @@
       </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr"/>
+      <c r="N17" s="7" t="inlineStr"/>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr"/>
-      <c r="E17" s="7" t="inlineStr"/>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M17" s="7" t="inlineStr">
+      <c r="M18" s="5" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N17" s="7" t="inlineStr">
+      <c r="N18" s="5" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="O18" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P17" s="7" t="inlineStr">
+      <c r="P18" s="5" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-28
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -104,10 +104,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P18" headerRowCount="1">
-  <autoFilter ref="A1:P18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P19" headerRowCount="1">
+  <autoFilter ref="A1:P19"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,173 +665,169 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>11756729075</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>85274983700047</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>REMIXT</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>75010</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 10</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>114533</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>https://remixt.co</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="inlineStr"/>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>site_sans_email</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-28 10:27:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
           <t>11921529392</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>48276116000019</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>ORSYS</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>92044</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>PUTEAUX</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>116153</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>1795</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>Spécialités plurivalentes des échanges et de la gestion</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>https://www.orsys.fr</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr">
         <is>
           <t>contactpresse@orsys.fr</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>contactpresse@orsys.fr;psh-accueil@orsys.fr;rgpd@orsys.fr</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>2026-10-27 09:42:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>11756068975</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>79935188700077</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>MARIANNE FORMATION</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>116400</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>2036</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>Enseignement, formation</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>https://marianne-education.fr</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>contact@marianne-education.fr</t>
-        </is>
-      </c>
-      <c r="M3" s="7" t="inlineStr">
-        <is>
-          <t>contact@marianne-education.fr</t>
-        </is>
-      </c>
-      <c r="N3" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P3" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-26 09:56:33</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11754723775</t>
+          <t>11756068975</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>53014903800719</t>
+          <t>79935188700077</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ENVERGURE</t>
+          <t>MARIANNE FORMATION</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr"/>
@@ -843,271 +839,287 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>116400</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>2036</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Enseignement, formation</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>https://marianne-education.fr</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>contact@marianne-education.fr</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>contact@marianne-education.fr</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:56:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>11754723775</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>53014903800719</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>ENVERGURE</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
           <t>formation;bilan;vae</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>118818</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>858</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>Formations générales</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>https://www.envergure.eu</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L5" s="7" t="inlineStr">
         <is>
           <t>jean.dupont@gmail.com</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>2026-10-24 08:46:35</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>53351042035</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>83923926600043</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>SIMANGO</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>35000</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>RENNES</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>119833</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Santé</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>https://simango.fr</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>contact@simango.fr</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr">
-        <is>
-          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
-        </is>
-      </c>
-      <c r="N5" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O5" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P5" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-23 09:13:07</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
+          <t>53351042035</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>83923926600043</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>SIMANGO</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>RENNES</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>119833</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Santé</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>https://simango.fr</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 09:13:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
           <t>28610102561</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>83411160100011</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>UDD</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>formation;vae</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>128484</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>2756</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>Linguistique</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>https://udd.eu</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr"/>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>site_sans_email</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>2026-10-22 09:17:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>31590340859</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>40073444800022</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>formation;apprentissage;bilan</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>129603</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>520</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
-      <c r="M7" s="7" t="inlineStr"/>
-      <c r="N7" s="7" t="inlineStr"/>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P7" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-21 09:14:55</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>22020084902</t>
+          <t>31590340859</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>39017462100404</t>
+          <t>40073444800022</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>AKSIS</t>
+          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr"/>
@@ -1119,274 +1131,270 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>formation;bilan</t>
+          <t>formation;apprentissage;bilan</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>142980</t>
+          <t>129603</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>https://www.aksis.fr</t>
-        </is>
-      </c>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr"/>
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr"/>
       <c r="N8" s="5" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr">
         <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 09:14:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>22020084902</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>39017462100404</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>formation;bilan</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>142980</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>707</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr"/>
+      <c r="N9" s="6" t="inlineStr"/>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
           <t>site_sans_email</t>
         </is>
       </c>
-      <c r="P8" s="5" t="inlineStr">
+      <c r="P9" s="6" t="inlineStr">
         <is>
           <t>2026-10-20 09:17:58</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>11753916975</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>47916313100119</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>147210</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>1043</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K9" s="7" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr"/>
-      <c r="M9" s="7" t="inlineStr"/>
-      <c r="N9" s="7" t="inlineStr"/>
-      <c r="O9" s="7" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P9" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-19 09:44:56</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>11753916975</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>47916313100119</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>147210</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>1043</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr"/>
+      <c r="M10" s="5" t="inlineStr"/>
+      <c r="N10" s="5" t="inlineStr"/>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-19 09:44:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
           <t>11788376778</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>83409674500197</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>SOCOTEC FORMATION</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>181212</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>1344</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>https://formation.socotec.fr</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="L11" s="7" t="inlineStr">
         <is>
           <t>formation@socotec.com</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>formation@socotec.com</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O10" s="5" t="inlineStr">
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P10" s="5" t="inlineStr">
+      <c r="P11" s="6" t="inlineStr">
         <is>
           <t>2026-10-17 08:24:44</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>76310894831</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>38347481400100</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>182662</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>377</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>Technologies industrielles fondamentales</t>
-        </is>
-      </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L11" s="7" t="inlineStr"/>
-      <c r="M11" s="7" t="inlineStr"/>
-      <c r="N11" s="7" t="inlineStr"/>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>site_sans_email</t>
-        </is>
-      </c>
-      <c r="P11" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1396,12 +1404,12 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -1411,7 +1419,7 @@
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr"/>
@@ -1424,441 +1432,503 @@
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
+          <t>2026-10-15 09:02:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>11750082675</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>56208290901190</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>SAFRAN</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>239038</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>Technologies industrielles fondamentales</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr"/>
+      <c r="M13" s="6" t="inlineStr"/>
+      <c r="N13" s="6" t="inlineStr"/>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>site_sans_email</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr">
+        <is>
           <t>2026-10-14 09:23:38</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>11920012692</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>55202467100091</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>CEGOS SA</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr"/>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>187508</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>1936</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="inlineStr">
-        <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L13" s="6" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M13" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P13" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>11920012692</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>55202467100091</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>187508</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>1936</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cegos.fr</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 09:23:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t>11750091675</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>30540504500017</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>AFTRAL</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>75847</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>PARIS 17</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>formation;apprentissage;vae</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>293734</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>2259</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Transport, manutention, magasinage</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>https://www.aftral.com</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="L15" s="7" t="inlineStr">
         <is>
           <t>dpd@aftral.com</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>dpd@aftral.com</t>
         </is>
       </c>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P14" s="5" t="inlineStr">
+      <c r="P15" s="6" t="inlineStr">
         <is>
           <t>2026-10-13 11:34:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>82690030969</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>95550398200014</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr"/>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>368655</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
-        </is>
-      </c>
-      <c r="K15" s="7" t="inlineStr">
-        <is>
-          <t>https://www.desautel.fr</t>
-        </is>
-      </c>
-      <c r="L15" s="6" t="inlineStr">
-        <is>
-          <t>contact@desautel.fr</t>
-        </is>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
-        </is>
-      </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O15" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P15" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>82690030969</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>95550398200014</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>368655</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12 11:47:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t>11756597175</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>80360838900026</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>75009</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>PARIS 09</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>426616</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>Formations générales</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr"/>
-      <c r="L16" s="5" t="inlineStr"/>
-      <c r="M16" s="5" t="inlineStr"/>
-      <c r="N16" s="5" t="inlineStr"/>
-      <c r="O16" s="5" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr"/>
+      <c r="N17" s="6" t="inlineStr"/>
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>introuvable</t>
         </is>
       </c>
-      <c r="P16" s="5" t="inlineStr">
+      <c r="P17" s="6" t="inlineStr">
         <is>
           <t>2026-10-10 10:30:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>11922496392</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>90386961800012</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>486807</t>
-        </is>
-      </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>2713</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t>Energie, génie climatique</t>
-        </is>
-      </c>
-      <c r="K17" s="7" t="inlineStr"/>
-      <c r="L17" s="7" t="inlineStr"/>
-      <c r="M17" s="7" t="inlineStr"/>
-      <c r="N17" s="7" t="inlineStr"/>
-      <c r="O17" s="7" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P17" s="7" t="inlineStr">
-        <is>
-          <t>2026-10-09 11:12:58</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr"/>
+      <c r="M18" s="5" t="inlineStr"/>
+      <c r="N18" s="5" t="inlineStr"/>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr"/>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="L19" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M18" s="5" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N18" s="5" t="inlineStr">
+      <c r="N19" s="6" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O18" s="5" t="inlineStr">
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P18" s="5" t="inlineStr">
+      <c r="P19" s="6" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-29
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -104,10 +104,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P19" headerRowCount="1">
-  <autoFilter ref="A1:P19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P20" headerRowCount="1">
+  <autoFilter ref="A1:P20"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,853 +665,865 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>82691041969</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>51012694900013</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>SOLERYS</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>formation;bilan</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>109484</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>710</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>https://solerys.fr</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>contact@solerys.fr</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>contact@solerys.fr</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:46:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
           <t>11756729075</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>85274983700047</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>REMIXT</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>75010</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>PARIS 10</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>114533</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Droit, sciences politiques</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>https://remixt.co</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
-      <c r="N2" s="5" t="inlineStr"/>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr"/>
+      <c r="M3" s="7" t="inlineStr"/>
+      <c r="N3" s="7" t="inlineStr"/>
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>site_sans_email</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>2026-10-28 10:27:20</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>11921529392</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>48276116000019</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>ORSYS</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>92044</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>PUTEAUX</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>116153</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>1795</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>Spécialités plurivalentes des échanges et de la gestion</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>https://www.orsys.fr</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>contactpresse@orsys.fr</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>contactpresse@orsys.fr;psh-accueil@orsys.fr;rgpd@orsys.fr</t>
-        </is>
-      </c>
-      <c r="N3" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O3" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P3" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-27 09:42:14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
+          <t>11921529392</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>48276116000019</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>ORSYS</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>92044</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>PUTEAUX</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>116153</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>1795</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Spécialités plurivalentes des échanges et de la gestion</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.orsys.fr</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>contactpresse@orsys.fr</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>contactpresse@orsys.fr;psh-accueil@orsys.fr;rgpd@orsys.fr</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-27 09:42:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
           <t>11756068975</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>79935188700077</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>MARIANNE FORMATION</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>116400</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>2036</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Enseignement, formation</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>https://marianne-education.fr</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>contact@marianne-education.fr</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M5" s="7" t="inlineStr">
         <is>
           <t>contact@marianne-education.fr</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N5" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O5" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>2026-10-26 09:56:33</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>11754723775</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>53014903800719</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>ENVERGURE</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>formation;bilan;vae</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>118818</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>858</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>https://www.envergure.eu</t>
-        </is>
-      </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>jean.dupont@gmail.com</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
-        </is>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O5" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P5" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-24 08:46:35</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
+          <t>11754723775</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>53014903800719</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>ENVERGURE</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>formation;bilan;vae</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>118818</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>858</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.envergure.eu</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>jean.dupont@gmail.com</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-24 08:46:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
           <t>53351042035</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>83923926600043</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>SIMANGO</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>35000</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>RENNES</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>53</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>119833</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>Santé</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>https://simango.fr</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>contact@simango.fr</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="N7" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O7" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="P7" s="7" t="inlineStr">
         <is>
           <t>2026-10-23 09:13:07</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>28610102561</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>83411160100011</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>UDD</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>formation;vae</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>128484</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>2756</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Linguistique</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>https://udd.eu</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr">
-        <is>
-          <t>site_sans_email</t>
-        </is>
-      </c>
-      <c r="P7" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-22 09:17:57</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>31590340859</t>
+          <t>28610102561</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>40073444800022</t>
+          <t>83411160100011</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr"/>
       <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>formation;apprentissage;bilan</t>
+          <t>formation;vae</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>129603</t>
+          <t>128484</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>2756</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr"/>
+          <t>Linguistique</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>https://udd.eu</t>
+        </is>
+      </c>
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr"/>
       <c r="N8" s="5" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr">
         <is>
+          <t>site_sans_email</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 09:17:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>31590340859</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>40073444800022</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>formation;apprentissage;bilan</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>129603</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>520</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr"/>
+      <c r="N9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
           <t>introuvable</t>
         </is>
       </c>
-      <c r="P8" s="5" t="inlineStr">
+      <c r="P9" s="7" t="inlineStr">
         <is>
           <t>2026-10-21 09:14:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>22020084902</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>39017462100404</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>AKSIS</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr"/>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>formation;bilan</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>142980</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>707</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>https://www.aksis.fr</t>
-        </is>
-      </c>
-      <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="6" t="inlineStr"/>
-      <c r="N9" s="6" t="inlineStr"/>
-      <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>site_sans_email</t>
-        </is>
-      </c>
-      <c r="P9" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-20 09:17:58</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>11753916975</t>
+          <t>22020084902</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>47916313100119</t>
+          <t>39017462100404</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>147210</t>
+          <t>142980</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>707</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr"/>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr"/>
       <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr">
         <is>
+          <t>site_sans_email</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20 09:17:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>11753916975</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>47916313100119</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>147210</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>1043</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr"/>
+      <c r="N11" s="7" t="inlineStr"/>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
           <t>introuvable</t>
         </is>
       </c>
-      <c r="P10" s="5" t="inlineStr">
+      <c r="P11" s="7" t="inlineStr">
         <is>
           <t>2026-10-19 09:44:56</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>11788376778</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>83409674500197</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>SOCOTEC FORMATION</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr"/>
-      <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>181212</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>1344</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>Electricité, électronique (non compris automatisme et productique)</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>https://formation.socotec.fr</t>
-        </is>
-      </c>
-      <c r="L11" s="7" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="N11" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O11" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P11" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-17 08:24:44</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
+          <t>11788376778</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>83409674500197</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>SOCOTEC FORMATION</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>181212</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>1344</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Electricité, électronique (non compris automatisme et productique)</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>https://formation.socotec.fr</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17 08:24:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
           <t>76310894831</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>38347481400100</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>AIRBUS SAS</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>31700</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>BLAGNAC</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>76</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>182662</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>377</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J13" s="7" t="inlineStr">
         <is>
           <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K13" s="7" t="inlineStr">
         <is>
           <t>https://www.airbus.com</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr"/>
-      <c r="M12" s="5" t="inlineStr"/>
-      <c r="N12" s="5" t="inlineStr"/>
-      <c r="O12" s="5" t="inlineStr">
+      <c r="L13" s="7" t="inlineStr"/>
+      <c r="M13" s="7" t="inlineStr"/>
+      <c r="N13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr">
         <is>
           <t>site_sans_email</t>
         </is>
       </c>
-      <c r="P12" s="5" t="inlineStr">
+      <c r="P13" s="7" t="inlineStr">
         <is>
           <t>2026-10-15 09:02:13</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>11750082675</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>56208290901190</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr"/>
-      <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>239038</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Technologies industrielles fondamentales</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>http://safran-formation.com</t>
-        </is>
-      </c>
-      <c r="L13" s="6" t="inlineStr"/>
-      <c r="M13" s="6" t="inlineStr"/>
-      <c r="N13" s="6" t="inlineStr"/>
-      <c r="O13" s="6" t="inlineStr">
-        <is>
-          <t>site_sans_email</t>
-        </is>
-      </c>
-      <c r="P13" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr"/>
@@ -1528,296 +1540,292 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
+          <t>239038</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Technologies industrielles fondamentales</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr"/>
+      <c r="M14" s="5" t="inlineStr"/>
+      <c r="N14" s="5" t="inlineStr"/>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>site_sans_email</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14 09:23:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>11920012692</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>55202467100091</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
           <t>187508</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>1936</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J15" s="7" t="inlineStr">
         <is>
           <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K15" s="7" t="inlineStr">
         <is>
           <t>https://www.cegos.fr</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>nomprenom@gmail.com</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="M15" s="7" t="inlineStr">
         <is>
           <t>nomprenom@gmail.com;dpo@cegos.fr</t>
         </is>
       </c>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="N15" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr">
+      <c r="O15" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P14" s="5" t="inlineStr">
+      <c r="P15" s="7" t="inlineStr">
         <is>
           <t>2026-10-14 09:23:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>11750091675</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>30540504500017</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>formation;apprentissage;vae</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>293734</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>2259</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>Transport, manutention, magasinage</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>https://www.aftral.com</t>
-        </is>
-      </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>dpd@aftral.com</t>
-        </is>
-      </c>
-      <c r="M15" s="6" t="inlineStr">
-        <is>
-          <t>dpd@aftral.com</t>
-        </is>
-      </c>
-      <c r="N15" s="6" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
-      <c r="O15" s="6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="P15" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>11750091675</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>30540504500017</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>formation;apprentissage;vae</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>293734</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>2259</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Transport, manutention, magasinage</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aftral.com</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>dpd@aftral.com</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>dpd@aftral.com</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13 11:34:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
           <t>82690030969</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>95550398200014</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>DESAUTEL</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr"/>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>formation</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>368655</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>56</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
         <is>
           <t>Sécurité des biens et des personnes, police, surveillance</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
         <is>
           <t>https://www.desautel.fr</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>contact@desautel.fr</t>
         </is>
       </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M17" s="7" t="inlineStr">
         <is>
           <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
         </is>
       </c>
-      <c r="N16" s="5" t="inlineStr">
+      <c r="N17" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O16" s="5" t="inlineStr">
+      <c r="O17" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P16" s="5" t="inlineStr">
+      <c r="P17" s="7" t="inlineStr">
         <is>
           <t>2026-10-12 11:47:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>11756597175</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>80360838900026</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>formation</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>426616</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="6" t="inlineStr"/>
-      <c r="O17" s="6" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="P17" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1832,17 +1840,17 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr"/>
@@ -1856,79 +1864,145 @@
       </c>
       <c r="P18" s="5" t="inlineStr">
         <is>
+          <t>2026-10-10 10:30:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr"/>
+      <c r="L19" s="7" t="inlineStr"/>
+      <c r="M19" s="7" t="inlineStr"/>
+      <c r="N19" s="7" t="inlineStr"/>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
           <t>2026-10-09 11:12:58</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L19" s="7" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="M20" s="5" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N19" s="6" t="inlineStr">
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr">
+      <c r="O20" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P19" s="6" t="inlineStr">
+      <c r="P20" s="5" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>

<commit_message>
🎓 Slice organismes de formation 2026-10-31
</commit_message>
<xml_diff>
--- a/exports/organismes_formation/organismes_formation.xlsx
+++ b/exports/organismes_formation/organismes_formation.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P20" headerRowCount="1">
-  <autoFilter ref="A1:P20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseOrganismesFormation" displayName="BaseOrganismesFormation" ref="A1:P21" headerRowCount="1">
+  <autoFilter ref="A1:P21"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nda"/>
     <tableColumn id="2" name="siret"/>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -665,59 +665,67 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>82691041969</t>
+          <t>11755666775</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>51012694900013</t>
+          <t>60206248102394</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>SOLERYS</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr"/>
-      <c r="E2" s="5" t="inlineStr"/>
+          <t>GENERALI VIE</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>PARIS 09</t>
+        </is>
+      </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>formation;bilan</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>109484</t>
+          <t>104169</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>710</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+          <t>Finances, banque, assurances</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>https://solerys.fr</t>
+          <t>https://www.generali.fr</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>contact@solerys.fr</t>
+          <t>droitdacces@generali.fr</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>contact@solerys.fr</t>
+          <t>droitdacces@generali.fr</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
@@ -732,104 +740,108 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 10:46:55</t>
+          <t>2026-10-31 10:16:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>11756729075</t>
+          <t>82691041969</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>85274983700047</t>
+          <t>51012694900013</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>REMIXT</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>75010</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>PARIS 10</t>
-        </is>
-      </c>
+          <t>SOLERYS</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>114533</t>
+          <t>109484</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>710</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Droit, sciences politiques</t>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>https://remixt.co</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr"/>
-      <c r="M3" s="7" t="inlineStr"/>
-      <c r="N3" s="7" t="inlineStr"/>
+          <t>https://solerys.fr</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>contact@solerys.fr</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>contact@solerys.fr</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P3" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 10:27:20</t>
+          <t>2026-10-29 10:46:55</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11921529392</t>
+          <t>11756729075</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>48276116000019</t>
+          <t>85274983700047</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ORSYS</t>
+          <t>REMIXT</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>92044</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>PUTEAUX</t>
+          <t>PARIS 10</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -844,68 +856,64 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>116153</t>
+          <t>114533</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>1795</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Spécialités plurivalentes des échanges et de la gestion</t>
+          <t>Droit, sciences politiques</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>https://www.orsys.fr</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>contactpresse@orsys.fr</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>contactpresse@orsys.fr;psh-accueil@orsys.fr;rgpd@orsys.fr</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>https://remixt.co</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
+      <c r="N4" s="5" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27 09:42:14</t>
+          <t>2026-10-28 10:27:20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>11756068975</t>
+          <t>11921529392</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>79935188700077</t>
+          <t>48276116000019</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>MARIANNE FORMATION</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
+          <t>ORSYS</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>92044</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>PUTEAUX</t>
+        </is>
+      </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
           <t>11</t>
@@ -918,32 +926,32 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>116400</t>
+          <t>116153</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>2036</t>
+          <t>1795</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Enseignement, formation</t>
+          <t>Spécialités plurivalentes des échanges et de la gestion</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>https://marianne-education.fr</t>
+          <t>https://www.orsys.fr</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>contact@marianne-education.fr</t>
+          <t>contactpresse@orsys.fr</t>
         </is>
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>contact@marianne-education.fr</t>
+          <t>contactpresse@orsys.fr;psh-accueil@orsys.fr;rgpd@orsys.fr</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
@@ -958,24 +966,24 @@
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>2026-10-26 09:56:33</t>
+          <t>2026-10-27 09:42:14</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>11754723775</t>
+          <t>11756068975</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>53014903800719</t>
+          <t>79935188700077</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ENVERGURE</t>
+          <t>MARIANNE FORMATION</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr"/>
@@ -987,37 +995,37 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>formation;bilan;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>118818</t>
+          <t>116400</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>858</t>
+          <t>2036</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
+          <t>Enseignement, formation</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>https://www.envergure.eu</t>
+          <t>https://marianne-education.fr</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>jean.dupont@gmail.com</t>
+          <t>contact@marianne-education.fr</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
+          <t>contact@marianne-education.fr</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -1032,74 +1040,66 @@
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24 08:46:35</t>
+          <t>2026-10-26 09:56:33</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>53351042035</t>
+          <t>11754723775</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>83923926600043</t>
+          <t>53014903800719</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>SIMANGO</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>35000</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>RENNES</t>
-        </is>
-      </c>
+          <t>ENVERGURE</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan;vae</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>119833</t>
+          <t>118818</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>858</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Santé</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>https://simango.fr</t>
+          <t>https://www.envergure.eu</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>contact@simango.fr</t>
+          <t>jean.dupont@gmail.com</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+          <t>jean.dupont@gmail.com;neil.graham@envergure.eu</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
@@ -1114,144 +1114,168 @@
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>2026-10-23 09:13:07</t>
+          <t>2026-10-24 08:46:35</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>28610102561</t>
+          <t>53351042035</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>83411160100011</t>
+          <t>83923926600043</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>UDD</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
+          <t>SIMANGO</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>RENNES</t>
+        </is>
+      </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>53</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>formation;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>128484</t>
+          <t>119833</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>2756</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Linguistique</t>
+          <t>Santé</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>https://udd.eu</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="inlineStr"/>
+          <t>https://simango.fr</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>handicap@simango.fr;communication@simango.fr;contact@simango.fr</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 09:17:57</t>
+          <t>2026-10-23 09:13:07</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>31590340859</t>
+          <t>28610102561</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>40073444800022</t>
+          <t>83411160100011</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
+          <t>UDD</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr"/>
       <c r="E9" s="7" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>formation;apprentissage;bilan</t>
+          <t>formation;vae</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>129603</t>
+          <t>128484</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>2756</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K9" s="7" t="inlineStr"/>
+          <t>Linguistique</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>https://udd.eu</t>
+        </is>
+      </c>
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr"/>
       <c r="N9" s="7" t="inlineStr"/>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-21 09:14:55</t>
+          <t>2026-10-22 09:17:57</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>22020084902</t>
+          <t>31590340859</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>39017462100404</t>
+          <t>40073444800022</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>AKSIS</t>
+          <t>INNOVATION DEVELOPT FORMATION I.D. FORMATION</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr"/>
@@ -1263,127 +1287,127 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>formation;bilan</t>
+          <t>formation;apprentissage;bilan</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>142980</t>
+          <t>129603</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>707</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>https://www.aksis.fr</t>
-        </is>
-      </c>
+          <t>Formations générales</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr"/>
       <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20 09:17:58</t>
+          <t>2026-10-21 09:14:55</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>11753916975</t>
+          <t>22020084902</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>47916313100119</t>
+          <t>39017462100404</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>LEFEBVRE DALLOZ COMPETENCES</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>92400</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>COURBEVOIE</t>
-        </is>
-      </c>
+          <t>AKSIS</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="inlineStr"/>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;bilan</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>147210</t>
+          <t>142980</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>1043</t>
+          <t>707</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Droit, sciences politiques</t>
-        </is>
-      </c>
-      <c r="K11" s="7" t="inlineStr"/>
+          <t>Développement des capacités d'orientation, d'insertion ou de réinsertion sociales et professionnelles</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>https://www.aksis.fr</t>
+        </is>
+      </c>
       <c r="L11" s="7" t="inlineStr"/>
       <c r="M11" s="7" t="inlineStr"/>
       <c r="N11" s="7" t="inlineStr"/>
       <c r="O11" s="7" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19 09:44:56</t>
+          <t>2026-10-20 09:17:58</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>11788376778</t>
+          <t>11753916975</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>83409674500197</t>
+          <t>47916313100119</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>SOCOTEC FORMATION</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr"/>
+          <t>LEFEBVRE DALLOZ COMPETENCES</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
           <t>11</t>
@@ -1396,79 +1420,55 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>181212</t>
+          <t>147210</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1043</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Electricité, électronique (non compris automatisme et productique)</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>https://formation.socotec.fr</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>formation@socotec.com</t>
-        </is>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>Droit, sciences politiques</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr"/>
+      <c r="M12" s="5" t="inlineStr"/>
+      <c r="N12" s="5" t="inlineStr"/>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17 08:24:44</t>
+          <t>2026-10-19 09:44:56</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>76310894831</t>
+          <t>11788376778</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>38347481400100</t>
+          <t>83409674500197</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>AIRBUS SAS</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>31700</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>BLAGNAC</t>
-        </is>
-      </c>
+          <t>SOCOTEC FORMATION</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="inlineStr"/>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1478,59 +1478,79 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>182662</t>
+          <t>181212</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Technologies industrielles fondamentales</t>
+          <t>Electricité, électronique (non compris automatisme et productique)</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>https://www.airbus.com</t>
-        </is>
-      </c>
-      <c r="L13" s="7" t="inlineStr"/>
-      <c r="M13" s="7" t="inlineStr"/>
-      <c r="N13" s="7" t="inlineStr"/>
+          <t>https://formation.socotec.fr</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>formation@socotec.com</t>
+        </is>
+      </c>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O13" s="7" t="inlineStr">
         <is>
-          <t>site_sans_email</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 09:02:13</t>
+          <t>2026-10-17 08:24:44</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>11750082675</t>
+          <t>76310894831</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>56208290901190</t>
+          <t>38347481400100</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>SAFRAN</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr"/>
-      <c r="E14" s="5" t="inlineStr"/>
+          <t>AIRBUS SAS</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>31700</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>BLAGNAC</t>
+        </is>
+      </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>76</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1540,12 +1560,12 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>239038</t>
+          <t>182662</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>377</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -1555,7 +1575,7 @@
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>http://safran-formation.com</t>
+          <t>https://www.airbus.com</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr"/>
@@ -1568,24 +1588,24 @@
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:38</t>
+          <t>2026-10-15 09:02:13</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>11920012692</t>
+          <t>11750082675</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>55202467100091</t>
+          <t>56208290901190</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>CEGOS SA</t>
+          <t>SAFRAN</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr"/>
@@ -1602,76 +1622,56 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>187508</t>
+          <t>239038</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
+          <t>Technologies industrielles fondamentales</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>https://www.cegos.fr</t>
-        </is>
-      </c>
-      <c r="L15" s="6" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com</t>
-        </is>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
-        </is>
-      </c>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>site</t>
-        </is>
-      </c>
+          <t>http://safran-formation.com</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr"/>
+      <c r="N15" s="7" t="inlineStr"/>
       <c r="O15" s="7" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>site_sans_email</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>2026-10-14 09:23:39</t>
+          <t>2026-10-14 09:23:38</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>11750091675</t>
+          <t>11920012692</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>30540504500017</t>
+          <t>55202467100091</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>AFTRAL</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>75847</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 17</t>
-        </is>
-      </c>
+          <t>CEGOS SA</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr"/>
       <c r="F16" s="5" t="inlineStr">
         <is>
           <t>11</t>
@@ -1679,37 +1679,37 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>formation;apprentissage;vae</t>
+          <t>formation</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>293734</t>
+          <t>187508</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Transport, manutention, magasinage</t>
+          <t>Ressources humaines, gestion du personnel, gestion de l'emploi</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>https://www.aftral.com</t>
+          <t>https://www.cegos.fr</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>dpd@aftral.com</t>
+          <t>nomprenom@gmail.com;dpo@cegos.fr</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
@@ -1724,66 +1724,74 @@
       </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13 11:34:14</t>
+          <t>2026-10-14 09:23:39</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>82690030969</t>
+          <t>11750091675</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>95550398200014</t>
+          <t>30540504500017</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>DESAUTEL</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr"/>
-      <c r="E17" s="7" t="inlineStr"/>
+          <t>AFTRAL</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>75847</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>PARIS 17</t>
+        </is>
+      </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>formation</t>
+          <t>formation;apprentissage;vae</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>368655</t>
+          <t>293734</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>2259</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>Sécurité des biens et des personnes, police, surveillance</t>
+          <t>Transport, manutention, magasinage</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
-          <t>https://www.desautel.fr</t>
+          <t>https://www.aftral.com</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>contact@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+          <t>dpd@aftral.com</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
@@ -1798,39 +1806,31 @@
       </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>2026-10-12 11:47:00</t>
+          <t>2026-10-13 11:34:14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>11756597175</t>
+          <t>82690030969</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>80360838900026</t>
+          <t>95550398200014</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>COORPACADEMY FRANCE</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>PARIS 09</t>
-        </is>
-      </c>
+          <t>DESAUTEL</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr"/>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1840,58 +1840,74 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>426616</t>
+          <t>368655</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Formations générales</t>
-        </is>
-      </c>
-      <c r="K18" s="5" t="inlineStr"/>
-      <c r="L18" s="5" t="inlineStr"/>
-      <c r="M18" s="5" t="inlineStr"/>
-      <c r="N18" s="5" t="inlineStr"/>
+          <t>Sécurité des biens et des personnes, police, surveillance</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.desautel.fr</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>contact@desautel.fr;paris-sud@desautel.fr;paris-ouest@desautel.fr;paris-centre@desautel.fr;paris-nord@desautel.fr;limoges@desautel.fr;poitiers@desautel.fr;rouen@desautel.fr;lyon-ouest@desautel.fr;lyon-est@desautel.fr;strasbourg@desautel.fr;clermont-ferrand@desautel.fr;lille@desautel.fr;nancy@desautel.fr;reims@desautel.fr;nantes@desautel.fr;saint-etienne@desautel.fr;grenoble@desautel.fr;tours@desautel.fr;rennes@desautel.fr;montpellier@desautel.fr;bordeaux@desautel.fr;toulouse@desautel.fr;besancon@desautel.fr;dijon@desautel.fr;caen@desautel.fr;marseille@desautel.fr;nice@desautel.fr</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="P18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10 10:30:20</t>
+          <t>2026-10-12 11:47:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>11922496392</t>
+          <t>11756597175</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>90386961800012</t>
+          <t>80360838900026</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>APAVE EXPLOITATION FRANCE</t>
+          <t>COORPACADEMY FRANCE</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>92400</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>COURBEVOIE</t>
+          <t>PARIS 09</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -1906,17 +1922,17 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>486807</t>
+          <t>426616</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>2713</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>Energie, génie climatique</t>
+          <t>Formations générales</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr"/>
@@ -1930,79 +1946,145 @@
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09 11:12:58</t>
+          <t>2026-10-10 10:30:20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>11922496392</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>90386961800012</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>APAVE EXPLOITATION FRANCE</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>92400</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>COURBEVOIE</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>formation</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>486807</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>2713</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Energie, génie climatique</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr"/>
+      <c r="M20" s="5" t="inlineStr"/>
+      <c r="N20" s="5" t="inlineStr"/>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>introuvable</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:12:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
           <t>42670251267</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>41988381400024</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>CAP COMPETENCES ACTIVATEUR DE TALENTS</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr"/>
+      <c r="E21" s="7" t="inlineStr"/>
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>formation;apprentissage</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>982270</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I21" s="7" t="inlineStr">
         <is>
           <t>8232</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>Finances, banque, assurances</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K21" s="7" t="inlineStr">
         <is>
           <t>https://capcompetences.eu</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="M21" s="7" t="inlineStr">
         <is>
           <t>contact@capcompetences.eu</t>
         </is>
       </c>
-      <c r="N20" s="5" t="inlineStr">
+      <c r="N21" s="7" t="inlineStr">
         <is>
           <t>site</t>
         </is>
       </c>
-      <c r="O20" s="5" t="inlineStr">
+      <c r="O21" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="P20" s="5" t="inlineStr">
+      <c r="P21" s="7" t="inlineStr">
         <is>
           <t>2026-10-08 11:14:03</t>
         </is>

</xml_diff>